<commit_message>
more updates and edits to pipeline documentation
</commit_message>
<xml_diff>
--- a/PipelineDocumentation/ini_templates_sample_data/SITEID1_Flags_YYYY.xlsx
+++ b/PipelineDocumentation/ini_templates_sample_data/SITEID1_Flags_YYYY.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rosie/Documents/Micromet/Lab_Website/ecoflux-lab.github.io/PipelineDocumentation/images/ini_files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rosie/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74780ECA-DB60-5C46-AE71-206DF2519983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1980695F-9DD8-4848-99B7-C8E285E928B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39660" yWindow="500" windowWidth="25700" windowHeight="15580" xr2:uid="{1CFF81EC-1561-F64F-987B-EF266FB34167}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" xr2:uid="{1CFF81EC-1561-F64F-987B-EF266FB34167}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
   <si>
     <t>% This file contains flags that can be used to block out time periods during the first stage cleaning. The first 4 rows are reserved for comments.</t>
   </si>
@@ -478,7 +478,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8722B469-F8CD-C146-B954-47812582A68A}">
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.33203125" style="1" customWidth="1"/>
@@ -554,27 +554,37 @@
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
+      <c r="A7" s="4">
+        <v>44668.708333333336</v>
+      </c>
+      <c r="B7" s="4">
+        <v>44668.791666666664</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7"/>
+      <c r="E7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
         <v>44805.416666666664</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B8" s="2">
         <v>44813.645833333336</v>
       </c>
-      <c r="C7"/>
-      <c r="D7">
+      <c r="C8"/>
+      <c r="D8">
         <v>1</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" s="4"/>
-      <c r="C8"/>
-      <c r="D8"/>
-      <c r="E8"/>
-    </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A9" s="4"/>
       <c r="C9"/>
       <c r="D9"/>
       <c r="E9"/>
@@ -615,7 +625,6 @@
       <c r="E16"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B17" s="1"/>
       <c r="C17"/>
       <c r="D17"/>
       <c r="E17"/>
@@ -651,7 +660,13 @@
       <c r="E22"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="5"/>
+      <c r="B23" s="1"/>
+      <c r="C23"/>
+      <c r="D23"/>
+      <c r="E23"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" s="5"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F1:H1 F2:J4">
@@ -664,7 +679,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K1:K4 F23:K1048576 C5:D22">
+  <conditionalFormatting sqref="K1:K4 C5:D23 F24:K1048576">
     <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
       <formula>1</formula>
     </cfRule>

</xml_diff>